<commit_message>
update: deuda interna — 381 new rows, total 4.42B USD (Sep 2026)
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 22-Aug-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 12-Sep-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1930761460.400001</v>
+        <v>1970002216.109999</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1314172597.270001</v>
+        <v>1350282301.89</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>48613140.7</v>
+        <v>51407640.21999999</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>24436753.44</v>
+        <v>24773305.01</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>28.15153400034169</v>
+        <v>27.5907795709632</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>68.06499012041293</v>
+        <v>68.54217172183141</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>2.51782220108789</v>
+        <v>2.609521948737215</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.265653678157496</v>
+        <v>1.257526758468211</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.672456521739131</v>
+        <v>7.74459457364341</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4379404303.27</v>
+        <v>4418645058.979999</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -909,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2375,19 +2375,44 @@
         </is>
       </c>
       <c r="C59" s="9" t="n">
-        <v>58115367.70999998</v>
+        <v>63187085.14999998</v>
       </c>
       <c r="D59" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="9" t="n">
-        <v>55021345.66999998</v>
+        <v>57353563.75999998</v>
       </c>
       <c r="F59" s="9" t="n">
-        <v>3094022.04</v>
+        <v>5833521.390000001</v>
       </c>
       <c r="G59" s="9" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>34169038.27000003</v>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>33777486.53000002</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>55000.17000000001</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>336551.57</v>
       </c>
     </row>
   </sheetData>
@@ -2404,7 +2429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3938,16 +3963,38 @@
         </is>
       </c>
       <c r="C70" s="7" t="n">
-        <v>5.9388</v>
+        <v>5.7535</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>7.8191</v>
+        <v>7.6667</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>8.4499</v>
+        <v>8.416499999999999</v>
       </c>
       <c r="F70" s="7" t="n">
-        <v>9.294499999999999</v>
+        <v>9.2264</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>4.8417</v>
+      </c>
+      <c r="D71" s="11" t="n">
+        <v>7.5018</v>
+      </c>
+      <c r="E71" s="11" t="n">
+        <v>8.331300000000001</v>
+      </c>
+      <c r="F71" s="11" t="n">
+        <v>9.047599999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3964,7 +4011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1273"/>
+  <dimension ref="A1:N1352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -72672,6 +72719,4272 @@
         </is>
       </c>
     </row>
+    <row r="1274">
+      <c r="A1274" s="23" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B1274" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1274" s="24" t="n">
+        <v>1049</v>
+      </c>
+      <c r="D1274" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1274" s="25" t="n">
+        <v>100.000012</v>
+      </c>
+      <c r="F1274" s="25" t="n">
+        <v>8.115500000000001</v>
+      </c>
+      <c r="G1274" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1274" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1274" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J1274" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1274" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1274" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1274" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1274" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="19" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B1275" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1275" s="20" t="n">
+        <v>1049</v>
+      </c>
+      <c r="D1275" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1275" s="21" t="n">
+        <v>100.000012</v>
+      </c>
+      <c r="F1275" s="21" t="n">
+        <v>8.115500000000001</v>
+      </c>
+      <c r="G1275" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1275" s="22" t="n">
+        <v>60000</v>
+      </c>
+      <c r="I1275" s="22" t="n">
+        <v>60000.01</v>
+      </c>
+      <c r="J1275" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1275" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1275" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1275" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1275" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="23" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B1276" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1276" s="24" t="n">
+        <v>1775</v>
+      </c>
+      <c r="D1276" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1276" s="25" t="n">
+        <v>100.000336</v>
+      </c>
+      <c r="F1276" s="25" t="n">
+        <v>8.2874</v>
+      </c>
+      <c r="G1276" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1276" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1276" s="26" t="n">
+        <v>15000.05</v>
+      </c>
+      <c r="J1276" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1276" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1276" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1276" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1276" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="19" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B1277" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1277" s="20" t="n">
+        <v>1049</v>
+      </c>
+      <c r="D1277" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1277" s="21" t="n">
+        <v>100.000012</v>
+      </c>
+      <c r="F1277" s="21" t="n">
+        <v>8.115500000000001</v>
+      </c>
+      <c r="G1277" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1277" s="22" t="n">
+        <v>92262</v>
+      </c>
+      <c r="I1277" s="22" t="n">
+        <v>92262.00999999999</v>
+      </c>
+      <c r="J1277" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1277" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1277" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1277" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1277" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="23" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B1278" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1278" s="24" t="n">
+        <v>1048</v>
+      </c>
+      <c r="D1278" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1278" s="25" t="n">
+        <v>100.00022</v>
+      </c>
+      <c r="F1278" s="25" t="n">
+        <v>8.1153</v>
+      </c>
+      <c r="G1278" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1278" s="26" t="n">
+        <v>360000</v>
+      </c>
+      <c r="I1278" s="26" t="n">
+        <v>360000.79</v>
+      </c>
+      <c r="J1278" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1278" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1278" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1278" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1278" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="19" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B1279" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1279" s="20" t="n">
+        <v>1048</v>
+      </c>
+      <c r="D1279" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1279" s="21" t="n">
+        <v>100.00022</v>
+      </c>
+      <c r="F1279" s="21" t="n">
+        <v>8.1153</v>
+      </c>
+      <c r="G1279" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1279" s="22" t="n">
+        <v>663000</v>
+      </c>
+      <c r="I1279" s="22" t="n">
+        <v>663001.46</v>
+      </c>
+      <c r="J1279" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1279" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1279" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1279" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1279" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="23" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B1280" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1280" s="24" t="n">
+        <v>1774</v>
+      </c>
+      <c r="D1280" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1280" s="25" t="n">
+        <v>99.99999800000001</v>
+      </c>
+      <c r="F1280" s="25" t="n">
+        <v>8.2874</v>
+      </c>
+      <c r="G1280" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1280" s="26" t="n">
+        <v>31000</v>
+      </c>
+      <c r="I1280" s="26" t="n">
+        <v>31000</v>
+      </c>
+      <c r="J1280" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1280" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1280" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1280" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1280" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="19" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B1281" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1281" s="20" t="n">
+        <v>1048</v>
+      </c>
+      <c r="D1281" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1281" s="21" t="n">
+        <v>100.00022</v>
+      </c>
+      <c r="F1281" s="21" t="n">
+        <v>8.1153</v>
+      </c>
+      <c r="G1281" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1281" s="22" t="n">
+        <v>83583</v>
+      </c>
+      <c r="I1281" s="22" t="n">
+        <v>83583.17999999999</v>
+      </c>
+      <c r="J1281" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1281" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1281" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1281" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1281" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="23" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B1282" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1282" s="24" t="n">
+        <v>1773</v>
+      </c>
+      <c r="D1282" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1282" s="25" t="n">
+        <v>100.000062</v>
+      </c>
+      <c r="F1282" s="25" t="n">
+        <v>8.2873</v>
+      </c>
+      <c r="G1282" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1282" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1282" s="26" t="n">
+        <v>1000000.62</v>
+      </c>
+      <c r="J1282" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1282" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1282" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1282" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1282" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="19" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B1283" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1283" s="20" t="n">
+        <v>1773</v>
+      </c>
+      <c r="D1283" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1283" s="21" t="n">
+        <v>100.000062</v>
+      </c>
+      <c r="F1283" s="21" t="n">
+        <v>8.2873</v>
+      </c>
+      <c r="G1283" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1283" s="22" t="n">
+        <v>118493</v>
+      </c>
+      <c r="I1283" s="22" t="n">
+        <v>118493.07</v>
+      </c>
+      <c r="J1283" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1283" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1283" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1283" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1283" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="23" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B1284" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1284" s="24" t="n">
+        <v>1046</v>
+      </c>
+      <c r="D1284" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1284" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1284" s="25" t="n">
+        <v>8.1151</v>
+      </c>
+      <c r="G1284" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1284" s="26" t="n">
+        <v>16000</v>
+      </c>
+      <c r="I1284" s="26" t="n">
+        <v>16000.02</v>
+      </c>
+      <c r="J1284" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1284" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1284" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1284" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1284" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="19" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B1285" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1285" s="20" t="n">
+        <v>1772</v>
+      </c>
+      <c r="D1285" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1285" s="21" t="n">
+        <v>100.000131</v>
+      </c>
+      <c r="F1285" s="21" t="n">
+        <v>8.2872</v>
+      </c>
+      <c r="G1285" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1285" s="22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1285" s="22" t="n">
+        <v>30000.04</v>
+      </c>
+      <c r="J1285" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1285" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1285" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1285" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1285" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="23" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B1286" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1286" s="24" t="n">
+        <v>1045</v>
+      </c>
+      <c r="D1286" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1286" s="25" t="n">
+        <v>100.000109</v>
+      </c>
+      <c r="F1286" s="25" t="n">
+        <v>8.115</v>
+      </c>
+      <c r="G1286" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1286" s="26" t="n">
+        <v>27630</v>
+      </c>
+      <c r="I1286" s="26" t="n">
+        <v>27630.03</v>
+      </c>
+      <c r="J1286" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1286" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1286" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1286" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1286" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="19" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B1287" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1287" s="20" t="n">
+        <v>1045</v>
+      </c>
+      <c r="D1287" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1287" s="21" t="n">
+        <v>100.000109</v>
+      </c>
+      <c r="F1287" s="21" t="n">
+        <v>8.115</v>
+      </c>
+      <c r="G1287" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1287" s="22" t="n">
+        <v>14740</v>
+      </c>
+      <c r="I1287" s="22" t="n">
+        <v>14740.02</v>
+      </c>
+      <c r="J1287" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1287" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1287" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1287" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1287" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="23" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B1288" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1288" s="24" t="n">
+        <v>1771</v>
+      </c>
+      <c r="D1288" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1288" s="25" t="n">
+        <v>100.000204</v>
+      </c>
+      <c r="F1288" s="25" t="n">
+        <v>8.287100000000001</v>
+      </c>
+      <c r="G1288" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1288" s="26" t="n">
+        <v>45000</v>
+      </c>
+      <c r="I1288" s="26" t="n">
+        <v>45000.09</v>
+      </c>
+      <c r="J1288" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1288" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1288" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1288" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1288" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="19" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B1289" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1289" s="20" t="n">
+        <v>1769</v>
+      </c>
+      <c r="D1289" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1289" s="21" t="n">
+        <v>100.000366</v>
+      </c>
+      <c r="F1289" s="21" t="n">
+        <v>8.286899999999999</v>
+      </c>
+      <c r="G1289" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1289" s="22" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I1289" s="22" t="n">
+        <v>400001.46</v>
+      </c>
+      <c r="J1289" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1289" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1289" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1289" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1289" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="23" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B1290" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1290" s="24" t="n">
+        <v>1769</v>
+      </c>
+      <c r="D1290" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1290" s="25" t="n">
+        <v>100.000366</v>
+      </c>
+      <c r="F1290" s="25" t="n">
+        <v>8.286899999999999</v>
+      </c>
+      <c r="G1290" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1290" s="26" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I1290" s="26" t="n">
+        <v>400001.46</v>
+      </c>
+      <c r="J1290" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1290" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1290" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1290" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1290" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="19" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B1291" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1291" s="20" t="n">
+        <v>1769</v>
+      </c>
+      <c r="D1291" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1291" s="21" t="n">
+        <v>100.000366</v>
+      </c>
+      <c r="F1291" s="21" t="n">
+        <v>8.286899999999999</v>
+      </c>
+      <c r="G1291" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1291" s="22" t="n">
+        <v>700000</v>
+      </c>
+      <c r="I1291" s="22" t="n">
+        <v>700002.5600000001</v>
+      </c>
+      <c r="J1291" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1291" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1291" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1291" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1291" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="23" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B1292" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1292" s="24" t="n">
+        <v>1043</v>
+      </c>
+      <c r="D1292" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1292" s="25" t="n">
+        <v>100.000057</v>
+      </c>
+      <c r="F1292" s="25" t="n">
+        <v>8.114800000000001</v>
+      </c>
+      <c r="G1292" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1292" s="26" t="n">
+        <v>600000</v>
+      </c>
+      <c r="I1292" s="26" t="n">
+        <v>600000.34</v>
+      </c>
+      <c r="J1292" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1292" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1292" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1292" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1292" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="19" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B1293" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1293" s="20" t="n">
+        <v>1043</v>
+      </c>
+      <c r="D1293" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1293" s="21" t="n">
+        <v>100.000057</v>
+      </c>
+      <c r="F1293" s="21" t="n">
+        <v>8.114800000000001</v>
+      </c>
+      <c r="G1293" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1293" s="22" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I1293" s="22" t="n">
+        <v>400000.23</v>
+      </c>
+      <c r="J1293" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1293" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1293" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1293" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1293" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="23" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1294" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1294" s="24" t="n">
+        <v>1042</v>
+      </c>
+      <c r="D1294" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1294" s="25" t="n">
+        <v>100.000038</v>
+      </c>
+      <c r="F1294" s="25" t="n">
+        <v>8.114699999999999</v>
+      </c>
+      <c r="G1294" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1294" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1294" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1294" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1294" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1294" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1294" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1294" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1295" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1295" s="20" t="n">
+        <v>1042</v>
+      </c>
+      <c r="D1295" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1295" s="21" t="n">
+        <v>100.000038</v>
+      </c>
+      <c r="F1295" s="21" t="n">
+        <v>8.114699999999999</v>
+      </c>
+      <c r="G1295" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1295" s="22" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I1295" s="22" t="n">
+        <v>7000</v>
+      </c>
+      <c r="J1295" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1295" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1295" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1295" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1295" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="23" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B1296" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1296" s="24" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D1296" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1296" s="25" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1296" s="25" t="n">
+        <v>8.114599999999999</v>
+      </c>
+      <c r="G1296" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1296" s="26" t="n">
+        <v>33600</v>
+      </c>
+      <c r="I1296" s="26" t="n">
+        <v>33600.01</v>
+      </c>
+      <c r="J1296" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1296" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1296" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1296" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1296" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="19" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B1297" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1297" s="20" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D1297" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1297" s="21" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1297" s="21" t="n">
+        <v>8.114599999999999</v>
+      </c>
+      <c r="G1297" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1297" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="I1297" s="22" t="n">
+        <v>1500000.34</v>
+      </c>
+      <c r="J1297" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1297" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1297" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1297" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1297" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="23" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B1298" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1298" s="24" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D1298" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1298" s="25" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1298" s="25" t="n">
+        <v>8.114599999999999</v>
+      </c>
+      <c r="G1298" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1298" s="26" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="I1298" s="26" t="n">
+        <v>1500000.34</v>
+      </c>
+      <c r="J1298" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1298" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1298" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1298" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1298" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="19" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B1299" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1299" s="20" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D1299" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1299" s="21" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1299" s="21" t="n">
+        <v>8.114599999999999</v>
+      </c>
+      <c r="G1299" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1299" s="22" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="I1299" s="22" t="n">
+        <v>1500000.34</v>
+      </c>
+      <c r="J1299" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1299" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1299" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1299" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1299" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="23" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1300" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1300" s="24" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D1300" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1300" s="25" t="n">
+        <v>100.000013</v>
+      </c>
+      <c r="F1300" s="25" t="n">
+        <v>8.1145</v>
+      </c>
+      <c r="G1300" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1300" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1300" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="J1300" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1300" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1300" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1300" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1300" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="19" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1301" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1301" s="20" t="n">
+        <v>2404</v>
+      </c>
+      <c r="D1301" s="15" t="inlineStr">
+        <is>
+          <t>Mas de 5</t>
+        </is>
+      </c>
+      <c r="E1301" s="21" t="n">
+        <v>100.000466</v>
+      </c>
+      <c r="F1301" s="21" t="n">
+        <v>8.366</v>
+      </c>
+      <c r="G1301" s="21" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="H1301" s="22" t="n">
+        <v>336550</v>
+      </c>
+      <c r="I1301" s="22" t="n">
+        <v>336551.57</v>
+      </c>
+      <c r="J1301" s="19" t="n">
+        <v>46149</v>
+      </c>
+      <c r="K1301" s="19" t="n">
+        <v>48706</v>
+      </c>
+      <c r="L1301" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1301" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1301" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="23" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1302" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1302" s="24" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D1302" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1302" s="25" t="n">
+        <v>100.000013</v>
+      </c>
+      <c r="F1302" s="25" t="n">
+        <v>8.1145</v>
+      </c>
+      <c r="G1302" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1302" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1302" s="26" t="n">
+        <v>500000.06</v>
+      </c>
+      <c r="J1302" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1302" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1302" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1302" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1302" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="19" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1303" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1303" s="20" t="n">
+        <v>1040</v>
+      </c>
+      <c r="D1303" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1303" s="21" t="n">
+        <v>100.000013</v>
+      </c>
+      <c r="F1303" s="21" t="n">
+        <v>8.1145</v>
+      </c>
+      <c r="G1303" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1303" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1303" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1303" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1303" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1303" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1303" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1303" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="23" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1304" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1304" s="24" t="n">
+        <v>1039</v>
+      </c>
+      <c r="D1304" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1304" s="25" t="n">
+        <v>100.000007</v>
+      </c>
+      <c r="F1304" s="25" t="n">
+        <v>8.1144</v>
+      </c>
+      <c r="G1304" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1304" s="26" t="n">
+        <v>3859202.92</v>
+      </c>
+      <c r="I1304" s="26" t="n">
+        <v>3859203.18</v>
+      </c>
+      <c r="J1304" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1304" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1304" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1304" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1304" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="19" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1305" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1305" s="20" t="n">
+        <v>1036</v>
+      </c>
+      <c r="D1305" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1305" s="21" t="n">
+        <v>100.000017</v>
+      </c>
+      <c r="F1305" s="21" t="n">
+        <v>8.114100000000001</v>
+      </c>
+      <c r="G1305" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1305" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1305" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J1305" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1305" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1305" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1305" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1305" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="23" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1306" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1306" s="24" t="n">
+        <v>1039</v>
+      </c>
+      <c r="D1306" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1306" s="25" t="n">
+        <v>100.000007</v>
+      </c>
+      <c r="F1306" s="25" t="n">
+        <v>8.1144</v>
+      </c>
+      <c r="G1306" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1306" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1306" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1306" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1306" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1306" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1306" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1306" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="19" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1307" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1307" s="20" t="n">
+        <v>1765</v>
+      </c>
+      <c r="D1307" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1307" s="21" t="n">
+        <v>100.00035</v>
+      </c>
+      <c r="F1307" s="21" t="n">
+        <v>8.2866</v>
+      </c>
+      <c r="G1307" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1307" s="22" t="n">
+        <v>43000</v>
+      </c>
+      <c r="I1307" s="22" t="n">
+        <v>43000.15</v>
+      </c>
+      <c r="J1307" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1307" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1307" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1307" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1307" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="23" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1308" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1308" s="24" t="n">
+        <v>1039</v>
+      </c>
+      <c r="D1308" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1308" s="25" t="n">
+        <v>100.000007</v>
+      </c>
+      <c r="F1308" s="25" t="n">
+        <v>8.1144</v>
+      </c>
+      <c r="G1308" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1308" s="26" t="n">
+        <v>800000</v>
+      </c>
+      <c r="I1308" s="26" t="n">
+        <v>800000.05</v>
+      </c>
+      <c r="J1308" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1308" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1308" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1308" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1308" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="19" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1309" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1309" s="20" t="n">
+        <v>1036</v>
+      </c>
+      <c r="D1309" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1309" s="21" t="n">
+        <v>100.000017</v>
+      </c>
+      <c r="F1309" s="21" t="n">
+        <v>8.114100000000001</v>
+      </c>
+      <c r="G1309" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1309" s="22" t="n">
+        <v>36550</v>
+      </c>
+      <c r="I1309" s="22" t="n">
+        <v>36550.01</v>
+      </c>
+      <c r="J1309" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1309" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1309" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1309" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1309" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1310" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1310" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1310" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1310" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1310" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1310" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1310" s="26" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="I1310" s="26" t="n">
+        <v>6500001.88</v>
+      </c>
+      <c r="J1310" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1310" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1310" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1310" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1310" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1311" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1311" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1311" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1311" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1311" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1311" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1311" s="22" t="n">
+        <v>9860</v>
+      </c>
+      <c r="I1311" s="22" t="n">
+        <v>9860</v>
+      </c>
+      <c r="J1311" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1311" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1311" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1311" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1311" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1312" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1312" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1312" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1312" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1312" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1312" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1312" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1312" s="26" t="n">
+        <v>30000.01</v>
+      </c>
+      <c r="J1312" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1312" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1312" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1312" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1312" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1313" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1313" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1313" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1313" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1313" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1313" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1313" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1313" s="22" t="n">
+        <v>100000.03</v>
+      </c>
+      <c r="J1313" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1313" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1313" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1313" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1313" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1314" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1314" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1314" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1314" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1314" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1314" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1314" s="26" t="n">
+        <v>17930</v>
+      </c>
+      <c r="I1314" s="26" t="n">
+        <v>17930.01</v>
+      </c>
+      <c r="J1314" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1314" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1314" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1314" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1314" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1315" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1315" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1315" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1315" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1315" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1315" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1315" s="22" t="n">
+        <v>1148289</v>
+      </c>
+      <c r="I1315" s="22" t="n">
+        <v>1148289.33</v>
+      </c>
+      <c r="J1315" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1315" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1315" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1315" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1315" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1316" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1316" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1316" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1316" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1316" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1316" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1316" s="26" t="n">
+        <v>70000</v>
+      </c>
+      <c r="I1316" s="26" t="n">
+        <v>70000.02</v>
+      </c>
+      <c r="J1316" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1316" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1316" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1316" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1316" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1317" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1317" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1317" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1317" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1317" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1317" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1317" s="22" t="n">
+        <v>15140</v>
+      </c>
+      <c r="I1317" s="22" t="n">
+        <v>15140</v>
+      </c>
+      <c r="J1317" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1317" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1317" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1317" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1317" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1318" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1318" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1318" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1318" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1318" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1318" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1318" s="26" t="n">
+        <v>14100</v>
+      </c>
+      <c r="I1318" s="26" t="n">
+        <v>14100</v>
+      </c>
+      <c r="J1318" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1318" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1318" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1318" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1318" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1319" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1319" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1319" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1319" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1319" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1319" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1319" s="22" t="n">
+        <v>54000</v>
+      </c>
+      <c r="I1319" s="22" t="n">
+        <v>54000.02</v>
+      </c>
+      <c r="J1319" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1319" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1319" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1319" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1319" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1320" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1320" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1320" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1320" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1320" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1320" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1320" s="26" t="n">
+        <v>76615</v>
+      </c>
+      <c r="I1320" s="26" t="n">
+        <v>76615.02</v>
+      </c>
+      <c r="J1320" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1320" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1320" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1320" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1320" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1321" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1321" s="20" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1321" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1321" s="21" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1321" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1321" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1321" s="22" t="n">
+        <v>54485</v>
+      </c>
+      <c r="I1321" s="22" t="n">
+        <v>54485.02</v>
+      </c>
+      <c r="J1321" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1321" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1321" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1321" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1321" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1322" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1322" s="24" t="n">
+        <v>1035</v>
+      </c>
+      <c r="D1322" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1322" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1322" s="25" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1322" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1322" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1322" s="26" t="n">
+        <v>30000.01</v>
+      </c>
+      <c r="J1322" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1322" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1322" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1322" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1322" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="19" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1323" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1323" s="20" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1323" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1323" s="21" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1323" s="21" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1323" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1323" s="22" t="n">
+        <v>31900</v>
+      </c>
+      <c r="I1323" s="22" t="n">
+        <v>31900.01</v>
+      </c>
+      <c r="J1323" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1323" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1323" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1323" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1323" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="23" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1324" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1324" s="24" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1324" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1324" s="25" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1324" s="25" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1324" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1324" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1324" s="26" t="n">
+        <v>15000.01</v>
+      </c>
+      <c r="J1324" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1324" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1324" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1324" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1324" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="19" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1325" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1325" s="20" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1325" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1325" s="21" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1325" s="21" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1325" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1325" s="22" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I1325" s="22" t="n">
+        <v>12000.01</v>
+      </c>
+      <c r="J1325" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1325" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1325" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1325" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1325" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="23" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1326" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1326" s="24" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1326" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1326" s="25" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1326" s="25" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1326" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1326" s="26" t="n">
+        <v>617229</v>
+      </c>
+      <c r="I1326" s="26" t="n">
+        <v>617229.28</v>
+      </c>
+      <c r="J1326" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1326" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1326" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1326" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1326" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="19" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1327" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1327" s="20" t="n">
+        <v>1760</v>
+      </c>
+      <c r="D1327" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1327" s="21" t="n">
+        <v>100.000142</v>
+      </c>
+      <c r="F1327" s="21" t="n">
+        <v>8.286300000000001</v>
+      </c>
+      <c r="G1327" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1327" s="22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I1327" s="22" t="n">
+        <v>6000.01</v>
+      </c>
+      <c r="J1327" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1327" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1327" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1327" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1327" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="23" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1328" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1328" s="24" t="n">
+        <v>1760</v>
+      </c>
+      <c r="D1328" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1328" s="25" t="n">
+        <v>100.000142</v>
+      </c>
+      <c r="F1328" s="25" t="n">
+        <v>8.286300000000001</v>
+      </c>
+      <c r="G1328" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1328" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I1328" s="26" t="n">
+        <v>6000.01</v>
+      </c>
+      <c r="J1328" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1328" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1328" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1328" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1328" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="19" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1329" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1329" s="20" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1329" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1329" s="21" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1329" s="21" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1329" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1329" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I1329" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J1329" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1329" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1329" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1329" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1329" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="23" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1330" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1330" s="24" t="n">
+        <v>1034</v>
+      </c>
+      <c r="D1330" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1330" s="25" t="n">
+        <v>100.000046</v>
+      </c>
+      <c r="F1330" s="25" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1330" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1330" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1330" s="26" t="n">
+        <v>30000.01</v>
+      </c>
+      <c r="J1330" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1330" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1330" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1330" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1330" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1331" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1331" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1331" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1331" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1331" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1331" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1331" s="22" t="n">
+        <v>9000</v>
+      </c>
+      <c r="I1331" s="22" t="n">
+        <v>9000.01</v>
+      </c>
+      <c r="J1331" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1331" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1331" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1331" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1331" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1332" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1332" s="24" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1332" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1332" s="25" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1332" s="25" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1332" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1332" s="26" t="n">
+        <v>348180</v>
+      </c>
+      <c r="I1332" s="26" t="n">
+        <v>348180.23</v>
+      </c>
+      <c r="J1332" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1332" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1332" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1332" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1332" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1333" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1333" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1333" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1333" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1333" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1333" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1333" s="22" t="n">
+        <v>764936</v>
+      </c>
+      <c r="I1333" s="22" t="n">
+        <v>764936.51</v>
+      </c>
+      <c r="J1333" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1333" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1333" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1333" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1333" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1334" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1334" s="24" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1334" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1334" s="25" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1334" s="25" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1334" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1334" s="26" t="n">
+        <v>425685</v>
+      </c>
+      <c r="I1334" s="26" t="n">
+        <v>425685.28</v>
+      </c>
+      <c r="J1334" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1334" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1334" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1334" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1334" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1335" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1335" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1335" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1335" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1335" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1335" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1335" s="22" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I1335" s="22" t="n">
+        <v>5000003.35</v>
+      </c>
+      <c r="J1335" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1335" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1335" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1335" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1335" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1336" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1336" s="24" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1336" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1336" s="25" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1336" s="25" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1336" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1336" s="26" t="n">
+        <v>39270</v>
+      </c>
+      <c r="I1336" s="26" t="n">
+        <v>39270.03</v>
+      </c>
+      <c r="J1336" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1336" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1336" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1336" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1336" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1337" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1337" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1337" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1337" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1337" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1337" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1337" s="22" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I1337" s="22" t="n">
+        <v>25000.02</v>
+      </c>
+      <c r="J1337" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1337" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1337" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1337" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1337" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1338" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1338" s="24" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1338" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1338" s="25" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1338" s="25" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1338" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1338" s="26" t="n">
+        <v>5855153.74</v>
+      </c>
+      <c r="I1338" s="26" t="n">
+        <v>5855157.66</v>
+      </c>
+      <c r="J1338" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1338" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1338" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1338" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1338" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1339" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1339" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1339" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1339" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1339" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1339" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1339" s="22" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1339" s="22" t="n">
+        <v>20000.01</v>
+      </c>
+      <c r="J1339" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1339" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1339" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1339" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1339" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1340" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1340" s="24" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1340" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1340" s="25" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1340" s="25" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1340" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1340" s="26" t="n">
+        <v>150000</v>
+      </c>
+      <c r="I1340" s="26" t="n">
+        <v>150000.1</v>
+      </c>
+      <c r="J1340" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1340" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1340" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1340" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1340" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1341" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1341" s="20" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D1341" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1341" s="21" t="n">
+        <v>100.000067</v>
+      </c>
+      <c r="F1341" s="21" t="n">
+        <v>8.113799999999999</v>
+      </c>
+      <c r="G1341" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1341" s="22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1341" s="22" t="n">
+        <v>30000.02</v>
+      </c>
+      <c r="J1341" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1341" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1341" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1341" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1341" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1342" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1342" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1342" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1342" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1342" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1342" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1342" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1342" s="26" t="n">
+        <v>50000.05</v>
+      </c>
+      <c r="J1342" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1342" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1342" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1342" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1342" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1343" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1343" s="20" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1343" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1343" s="21" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1343" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1343" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1343" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1343" s="22" t="n">
+        <v>10000.01</v>
+      </c>
+      <c r="J1343" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1343" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1343" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1343" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1343" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1344" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1344" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1344" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1344" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1344" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1344" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1344" s="26" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I1344" s="26" t="n">
+        <v>8000.01</v>
+      </c>
+      <c r="J1344" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1344" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1344" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1344" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1344" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1345" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1345" s="20" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1345" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1345" s="21" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1345" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1345" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1345" s="22" t="n">
+        <v>517135</v>
+      </c>
+      <c r="I1345" s="22" t="n">
+        <v>517135.48</v>
+      </c>
+      <c r="J1345" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1345" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1345" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1345" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1345" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1346" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1346" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1346" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1346" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1346" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1346" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1346" s="26" t="n">
+        <v>374046</v>
+      </c>
+      <c r="I1346" s="26" t="n">
+        <v>374046.35</v>
+      </c>
+      <c r="J1346" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1346" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1346" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1346" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1346" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1347" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1347" s="20" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1347" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1347" s="21" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1347" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1347" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1347" s="22" t="n">
+        <v>102955</v>
+      </c>
+      <c r="I1347" s="22" t="n">
+        <v>102955.1</v>
+      </c>
+      <c r="J1347" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1347" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1347" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1347" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1347" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1348" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1348" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1348" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1348" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1348" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1348" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1348" s="26" t="n">
+        <v>259010</v>
+      </c>
+      <c r="I1348" s="26" t="n">
+        <v>259010.24</v>
+      </c>
+      <c r="J1348" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1348" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1348" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1348" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1348" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1349" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1349" s="20" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1349" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1349" s="21" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1349" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1349" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1349" s="22" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1349" s="22" t="n">
+        <v>1000000.93</v>
+      </c>
+      <c r="J1349" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1349" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1349" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1349" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1349" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1350" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1350" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1350" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1350" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1350" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1350" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1350" s="26" t="n">
+        <v>70200</v>
+      </c>
+      <c r="I1350" s="26" t="n">
+        <v>70200.07000000001</v>
+      </c>
+      <c r="J1350" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1350" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1350" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1350" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1350" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1351" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1351" s="20" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1351" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1351" s="21" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1351" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1351" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1351" s="22" t="n">
+        <v>70000</v>
+      </c>
+      <c r="I1351" s="22" t="n">
+        <v>70000.06</v>
+      </c>
+      <c r="J1351" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1351" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1351" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1351" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1351" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1352" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1352" s="24" t="n">
+        <v>1032</v>
+      </c>
+      <c r="D1352" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1352" s="25" t="n">
+        <v>100.000093</v>
+      </c>
+      <c r="F1352" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1352" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1352" s="26" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I1352" s="26" t="n">
+        <v>7000.01</v>
+      </c>
+      <c r="J1352" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1352" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1352" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1352" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1352" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
update: deuda interna — 146 new rows, total 4.50B USD (Oct 2026)
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09-Oct-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 20-Oct-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2021679208.999999</v>
+        <v>2053441209.959998</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1398659374.819999</v>
+        <v>1430409375.759999</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>54707560.17999998</v>
+        <v>54719560.19999999</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>24773305.01</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>26.88552004543073</v>
+        <v>26.46966303946868</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>69.1830518211557</v>
+        <v>69.65913456990882</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>2.706045545527497</v>
+        <v>2.664773646042974</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.225382587886129</v>
+        <v>1.206428744579573</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.79295501618123</v>
+        <v>7.79986609375</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4470322051.869998</v>
+        <v>4502084052.829998</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -2425,16 +2425,16 @@
         </is>
       </c>
       <c r="C61" s="9" t="n">
-        <v>17383244.98</v>
+        <v>49145245.94</v>
       </c>
       <c r="D61" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="9" t="n">
-        <v>17283244.87</v>
+        <v>49033245.80999999</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>100000.11</v>
+        <v>112000.13</v>
       </c>
       <c r="G61" s="9" t="n">
         <v>0</v>
@@ -4032,16 +4032,16 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>5</v>
+        <v>5.4837</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>7.7685</v>
+        <v>7.5379</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8.2723</v>
+        <v>8.293900000000001</v>
       </c>
       <c r="F72" s="7" t="n">
-        <v>9</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -4058,7 +4058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1454"/>
+  <dimension ref="A1:N1476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82540,6 +82540,1194 @@
         </is>
       </c>
     </row>
+    <row r="1455">
+      <c r="A1455" s="19" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1455" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1455" s="20" t="n">
+        <v>1001</v>
+      </c>
+      <c r="D1455" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1455" s="21" t="n">
+        <v>100.000193</v>
+      </c>
+      <c r="F1455" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1455" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1455" s="22" t="n">
+        <v>29400</v>
+      </c>
+      <c r="I1455" s="22" t="n">
+        <v>29400.06</v>
+      </c>
+      <c r="J1455" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1455" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1455" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1455" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1455" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="23" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1456" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1456" s="24" t="n">
+        <v>1001</v>
+      </c>
+      <c r="D1456" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1456" s="25" t="n">
+        <v>100.000193</v>
+      </c>
+      <c r="F1456" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1456" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1456" s="26" t="n">
+        <v>14900</v>
+      </c>
+      <c r="I1456" s="26" t="n">
+        <v>14900.03</v>
+      </c>
+      <c r="J1456" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1456" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1456" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1456" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1456" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="19" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1457" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1457" s="20" t="n">
+        <v>645</v>
+      </c>
+      <c r="D1457" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1457" s="21" t="n">
+        <v>100.000104</v>
+      </c>
+      <c r="F1457" s="21" t="n">
+        <v>7.1906</v>
+      </c>
+      <c r="G1457" s="21" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1457" s="22" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I1457" s="22" t="n">
+        <v>400000.42</v>
+      </c>
+      <c r="J1457" s="19" t="n">
+        <v>46230</v>
+      </c>
+      <c r="K1457" s="19" t="n">
+        <v>46961</v>
+      </c>
+      <c r="L1457" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1457" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1457" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="23" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1458" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1458" s="24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1458" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1458" s="25" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1458" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1458" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1458" s="26" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="I1458" s="26" t="n">
+        <v>2000002.43</v>
+      </c>
+      <c r="J1458" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1458" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1458" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1458" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1458" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1459" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1459" s="20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1459" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1459" s="21" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1459" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1459" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1459" s="22" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="I1459" s="22" t="n">
+        <v>6000007.28</v>
+      </c>
+      <c r="J1459" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1459" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1459" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1459" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1459" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="23" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1460" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1460" s="24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1460" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1460" s="25" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1460" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1460" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1460" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1460" s="26" t="n">
+        <v>500000.61</v>
+      </c>
+      <c r="J1460" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1460" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1460" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1460" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1460" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1461" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1461" s="20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1461" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1461" s="21" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1461" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1461" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1461" s="22" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="I1461" s="22" t="n">
+        <v>1300001.58</v>
+      </c>
+      <c r="J1461" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1461" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1461" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1461" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1461" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="23" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1462" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1462" s="24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1462" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1462" s="25" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1462" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1462" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1462" s="26" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="I1462" s="26" t="n">
+        <v>1100001.33</v>
+      </c>
+      <c r="J1462" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1462" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1462" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1462" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1462" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1463" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1463" s="20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1463" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1463" s="21" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1463" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1463" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1463" s="22" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="I1463" s="22" t="n">
+        <v>1100001.33</v>
+      </c>
+      <c r="J1463" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1463" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1463" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1463" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1463" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="23" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1464" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1464" s="24" t="n">
+        <v>644</v>
+      </c>
+      <c r="D1464" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1464" s="25" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1464" s="25" t="n">
+        <v>7.1906</v>
+      </c>
+      <c r="G1464" s="25" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1464" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1464" s="26" t="n">
+        <v>50000.01</v>
+      </c>
+      <c r="J1464" s="23" t="n">
+        <v>46230</v>
+      </c>
+      <c r="K1464" s="23" t="n">
+        <v>46961</v>
+      </c>
+      <c r="L1464" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1464" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1464" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="19" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1465" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1465" s="20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D1465" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1465" s="21" t="n">
+        <v>100.000121</v>
+      </c>
+      <c r="F1465" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1465" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1465" s="22" t="n">
+        <v>2066779.4</v>
+      </c>
+      <c r="I1465" s="22" t="n">
+        <v>2066781.91</v>
+      </c>
+      <c r="J1465" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1465" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1465" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1465" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1465" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="23" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1466" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1466" s="24" t="n">
+        <v>1725</v>
+      </c>
+      <c r="D1466" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1466" s="25" t="n">
+        <v>100.000193</v>
+      </c>
+      <c r="F1466" s="25" t="n">
+        <v>8.284700000000001</v>
+      </c>
+      <c r="G1466" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1466" s="26" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I1466" s="26" t="n">
+        <v>12000.02</v>
+      </c>
+      <c r="J1466" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1466" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1466" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1466" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1466" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1467" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1467" s="20" t="n">
+        <v>999</v>
+      </c>
+      <c r="D1467" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1467" s="21" t="n">
+        <v>100.000055</v>
+      </c>
+      <c r="F1467" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1467" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1467" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1467" s="22" t="n">
+        <v>15000.01</v>
+      </c>
+      <c r="J1467" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1467" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1467" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1467" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1467" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="23" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1468" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1468" s="24" t="n">
+        <v>999</v>
+      </c>
+      <c r="D1468" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1468" s="25" t="n">
+        <v>100.000055</v>
+      </c>
+      <c r="F1468" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1468" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1468" s="26" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I1468" s="26" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J1468" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1468" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1468" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1468" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1468" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1469" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1469" s="20" t="n">
+        <v>998</v>
+      </c>
+      <c r="D1469" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1469" s="21" t="n">
+        <v>100.000237</v>
+      </c>
+      <c r="F1469" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1469" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1469" s="22" t="n">
+        <v>58750</v>
+      </c>
+      <c r="I1469" s="22" t="n">
+        <v>58750.14</v>
+      </c>
+      <c r="J1469" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1469" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1469" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1469" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1469" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="23" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1470" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1470" s="24" t="n">
+        <v>998</v>
+      </c>
+      <c r="D1470" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1470" s="25" t="n">
+        <v>100.000237</v>
+      </c>
+      <c r="F1470" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1470" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1470" s="26" t="n">
+        <v>31140</v>
+      </c>
+      <c r="I1470" s="26" t="n">
+        <v>31140.07</v>
+      </c>
+      <c r="J1470" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1470" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1470" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1470" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1470" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1471" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1471" s="20" t="n">
+        <v>642</v>
+      </c>
+      <c r="D1471" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1471" s="21" t="n">
+        <v>100.000039</v>
+      </c>
+      <c r="F1471" s="21" t="n">
+        <v>7.1905</v>
+      </c>
+      <c r="G1471" s="21" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1471" s="22" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="I1471" s="22" t="n">
+        <v>7000002.74</v>
+      </c>
+      <c r="J1471" s="19" t="n">
+        <v>46230</v>
+      </c>
+      <c r="K1471" s="19" t="n">
+        <v>46961</v>
+      </c>
+      <c r="L1471" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1471" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1471" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="23" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1472" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1472" s="24" t="n">
+        <v>998</v>
+      </c>
+      <c r="D1472" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1472" s="25" t="n">
+        <v>100.000237</v>
+      </c>
+      <c r="F1472" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1472" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1472" s="26" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I1472" s="26" t="n">
+        <v>5000011.85</v>
+      </c>
+      <c r="J1472" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1472" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1472" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1472" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1472" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="19" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1473" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1473" s="20" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1473" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1473" s="21" t="n">
+        <v>100.00018</v>
+      </c>
+      <c r="F1473" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1473" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1473" s="22" t="n">
+        <v>19540</v>
+      </c>
+      <c r="I1473" s="22" t="n">
+        <v>19540.04</v>
+      </c>
+      <c r="J1473" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1473" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1473" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1473" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1473" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="23" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1474" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1474" s="24" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1474" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1474" s="25" t="n">
+        <v>100.00018</v>
+      </c>
+      <c r="F1474" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1474" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1474" s="26" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I1474" s="26" t="n">
+        <v>5000009</v>
+      </c>
+      <c r="J1474" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1474" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1474" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1474" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1474" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="19" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1475" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1475" s="20" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1475" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1475" s="21" t="n">
+        <v>100.00018</v>
+      </c>
+      <c r="F1475" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1475" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1475" s="22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1475" s="22" t="n">
+        <v>30000.05</v>
+      </c>
+      <c r="J1475" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1475" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1475" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1475" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1475" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="23" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1476" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1476" s="24" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1476" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1476" s="25" t="n">
+        <v>100.00018</v>
+      </c>
+      <c r="F1476" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1476" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1476" s="26" t="n">
+        <v>26450</v>
+      </c>
+      <c r="I1476" s="26" t="n">
+        <v>26450.05</v>
+      </c>
+      <c r="J1476" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1476" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1476" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1476" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1476" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>